<commit_message>
Update all outputs, models, and DB with cleaned schema results
- Schema: 68 rows x 138 cols (was 27 rows, +152% more data)
- Models: 5 targets trained, best R2=0.995 (Plant_Height_cm)
- New model: best_model_Yield_per_Hectare.pkl (R2=0.82)
- New file: feature_importance_Yield_per_Hectare.csv
- Features: 68 rows x 146 cols (was 27 rows)
- Recommendations: 11 crop-specific fertilizer recs
- Fuzzy rules: 221 rules (v3.0, expanded from 534 to 6819 lines)
- DB: 105 papers registered in paper_registry.sqlite
- Validated extractions: 6150+ lines of structured data
</commit_message>
<xml_diff>
--- a/outputs/Ready_Reckoner.xlsx
+++ b/outputs/Ready_Reckoner.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J73"/>
+  <dimension ref="A1:J114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2361,7 +2361,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Chickpea</t>
+          <t>Barley</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2376,7 +2376,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>, Rain 632.0mm</t>
+          <t>, Rain 355.0mm</t>
         </is>
       </c>
       <c r="E47" t="inlineStr"/>
@@ -2392,7 +2392,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Every 25-30 days</t>
+          <t>Every 15-20 days</t>
         </is>
       </c>
       <c r="I47" t="n">
@@ -2407,33 +2407,33 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Barley</t>
+          <t>Chickpea</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>MOP (Potassium-rich)</t>
+          <t>Balanced NPK (15-15-15)</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>pH 7.8, K 2.0</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>, Rain 683.0mm</t>
+          <t>, Rain 632.0mm</t>
         </is>
       </c>
       <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
         <is>
-          <t>MOP (Potassium-rich)</t>
+          <t>Balanced NPK (15-15-15)</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Soil application</t>
+          <t>Broadcast + incorporation</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2442,11 +2442,11 @@
         </is>
       </c>
       <c r="I48" t="n">
-        <v>0.65</v>
+        <v>0.75</v>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Increase potassium</t>
+          <t>Maintain current balanced fertilization</t>
         </is>
       </c>
     </row>
@@ -2466,11 +2466,7 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>, Rain 785.0mm</t>
-        </is>
-      </c>
+      <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
@@ -2499,7 +2495,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Barley</t>
+          <t>Chickpea</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2513,9 +2509,7 @@
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
-      <c r="E50" t="n">
-        <v>37.95</v>
-      </c>
+      <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
           <t>Balanced NPK (15-15-15)</t>
@@ -2543,33 +2537,33 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Barley</t>
+          <t>Black Wheat</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Balanced NPK (15-15-15)</t>
+          <t>DAP (Phosphorus-rich)</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>N/A, P 10.1, K 165.6</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>, Rain 502.0mm</t>
+          <t>, Rain 600.0mm</t>
         </is>
       </c>
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Balanced NPK (15-15-15)</t>
+          <t>DAP (Phosphorus-rich)</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Broadcast + incorporation</t>
+          <t>Soil application at sowing</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -2578,11 +2572,11 @@
         </is>
       </c>
       <c r="I51" t="n">
-        <v>0.75</v>
+        <v>0.65</v>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>Maintain current balanced fertilization</t>
+          <t>Increase phosphorus</t>
         </is>
       </c>
     </row>
@@ -2594,24 +2588,28 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Balanced NPK (15-15-15)</t>
+          <t>MOP (Potassium-rich)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr"/>
+          <t>pH 7.8, K 2.0</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>, Rain 683.0mm</t>
+        </is>
+      </c>
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Balanced NPK (15-15-15)</t>
+          <t>MOP (Potassium-rich)</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Broadcast + incorporation</t>
+          <t>Soil application</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -2620,18 +2618,18 @@
         </is>
       </c>
       <c r="I52" t="n">
-        <v>0.75</v>
+        <v>0.65</v>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>Maintain current balanced fertilization</t>
+          <t>Increase potassium</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Black Wheat</t>
+          <t>Barley</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2646,7 +2644,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>, Rain 651.0mm</t>
+          <t>, Rain 954.0mm</t>
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
@@ -2677,7 +2675,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Black Wheat</t>
+          <t>Chickpea</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2690,10 +2688,12 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="n">
-        <v>0.87</v>
-      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>, Rain 1431.0mm</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr">
         <is>
           <t>Balanced NPK (15-15-15)</t>
@@ -2706,7 +2706,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Every 25-30 days</t>
+          <t>Split application (3-4 splits)</t>
         </is>
       </c>
       <c r="I54" t="n">
@@ -2721,38 +2721,38 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Black Wheat</t>
+          <t>Barley</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Ammonium Sulphate + Gypsum</t>
+          <t>Balanced NPK (15-15-15)</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>pH 8.1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>, Rain 354.0mm</t>
+          <t>, Rain 542.0mm</t>
         </is>
       </c>
       <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Ammonium Sulphate + Gypsum</t>
+          <t>Balanced NPK (15-15-15)</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Soil application</t>
+          <t>Broadcast + incorporation</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Every 15-20 days</t>
+          <t>Every 25-30 days</t>
         </is>
       </c>
       <c r="I55" t="n">
@@ -2760,7 +2760,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>Apply sulfur-based amendments to reduce pH</t>
+          <t>Maintain current balanced fertilization</t>
         </is>
       </c>
     </row>
@@ -2813,7 +2813,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Chickpea</t>
+          <t>Barley</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2826,11 +2826,7 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>, Rain 1200.0mm</t>
-        </is>
-      </c>
+      <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr">
         <is>
@@ -2844,7 +2840,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Split application (3-4 splits)</t>
+          <t>Every 25-30 days</t>
         </is>
       </c>
       <c r="I57" t="n">
@@ -2859,7 +2855,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Bell Pepper</t>
+          <t>Chickpea</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2874,7 +2870,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>, Rain 16.5mm</t>
+          <t>, Rain 1200.0mm</t>
         </is>
       </c>
       <c r="E58" t="inlineStr"/>
@@ -2890,7 +2886,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>Every 15-20 days</t>
+          <t>Split application (3-4 splits)</t>
         </is>
       </c>
       <c r="I58" t="n">
@@ -2905,7 +2901,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Black Wheat</t>
+          <t>Barley</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2915,17 +2911,15 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>N/A, OC 4.0%</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>, Rain 48.0mm</t>
-        </is>
-      </c>
-      <c r="E59" t="n">
-        <v>5.46</v>
-      </c>
+          <t>, Rain 350.0mm</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr">
         <is>
           <t>Balanced NPK (15-15-15)</t>
@@ -2966,12 +2960,10 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>, Rain 355.0mm</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr"/>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="n">
+        <v>276</v>
+      </c>
       <c r="F60" t="inlineStr">
         <is>
           <t>Balanced NPK (15-15-15)</t>
@@ -2984,7 +2976,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>Every 15-20 days</t>
+          <t>Every 25-30 days</t>
         </is>
       </c>
       <c r="I60" t="n">
@@ -2999,7 +2991,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Black Wheat</t>
+          <t>Chickpea</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3009,10 +3001,14 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr"/>
+          <t>pH 5.53</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>, Rain 575.0mm</t>
+        </is>
+      </c>
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
         <is>
@@ -3041,72 +3037,66 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Black Wheat</t>
+          <t>Chickpea</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>MOP (Potassium-rich)</t>
+          <t>Balanced NPK (15-15-15)</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>N/A, P 20.0, K 5.0</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>, Rain 100.0mm</t>
-        </is>
-      </c>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
-          <t>MOP (Potassium-rich)</t>
+          <t>Balanced NPK (15-15-15)</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Soil application</t>
+          <t>Broadcast + incorporation</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>Every 15-20 days</t>
+          <t>Every 25-30 days</t>
         </is>
       </c>
       <c r="I62" t="n">
-        <v>0.65</v>
+        <v>0.75</v>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>Increase potassium</t>
+          <t>Maintain current balanced fertilization</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Black Wheat</t>
+          <t>Barley</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Dolomite + Bio NPK</t>
+          <t>Balanced NPK (15-15-15)</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>pH 5.0</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
-      <c r="E63" t="n">
-        <v>38.18</v>
-      </c>
+      <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Dolomite + Bio NPK</t>
+          <t>Balanced NPK (15-15-15)</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -3124,7 +3114,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>Apply lime to correct pH, then balanced NPK</t>
+          <t>Maintain current balanced fertilization</t>
         </is>
       </c>
     </row>
@@ -3173,28 +3163,24 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Barley</t>
+          <t>Black Wheat</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Balanced NPK (15-15-15)</t>
+          <t>Dolomite + Bio NPK</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>, Rain 542.0mm</t>
-        </is>
-      </c>
+          <t>pH 3.75</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Balanced NPK (15-15-15)</t>
+          <t>Dolomite + Bio NPK</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -3212,14 +3198,14 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>Maintain current balanced fertilization</t>
+          <t>Apply lime to correct pH, then balanced NPK</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Black Wheat</t>
+          <t>Barley</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3229,12 +3215,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>pH 7.7, OC 1.0%</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>, Rain 146.0mm</t>
+          <t>, Rain 55.0mm</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
@@ -3270,23 +3256,23 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Balanced NPK (15-15-15)</t>
+          <t>Compost + Vermicompost</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>N/A, OC 0.2003%</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>, Rain 954.0mm</t>
+          <t>, Rain 16.0mm</t>
         </is>
       </c>
       <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Balanced NPK (15-15-15)</t>
+          <t>Compost + Vermicompost</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -3296,7 +3282,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>Every 25-30 days</t>
+          <t>Every 15-20 days</t>
         </is>
       </c>
       <c r="I67" t="n">
@@ -3304,7 +3290,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>Maintain current balanced fertilization</t>
+          <t>Increase organic matter, apply slow-release fertilizer</t>
         </is>
       </c>
     </row>
@@ -3326,10 +3312,12 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>, Rain 10.0mm</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr"/>
+          <t>, Rain 700.0mm</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>9.199999999999999</v>
+      </c>
       <c r="F68" t="inlineStr">
         <is>
           <t>Balanced NPK (15-15-15)</t>
@@ -3342,7 +3330,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>Every 15-20 days</t>
+          <t>Every 25-30 days</t>
         </is>
       </c>
       <c r="I68" t="n">
@@ -3357,7 +3345,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Chickpea</t>
+          <t>Black Wheat</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3372,7 +3360,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>, Rain 0.0mm</t>
+          <t>, Rain 747.0mm</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
@@ -3388,7 +3376,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>Every 15-20 days</t>
+          <t>Every 25-30 days</t>
         </is>
       </c>
       <c r="I69" t="n">
@@ -3403,33 +3391,33 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Chickpea</t>
+          <t>Black Wheat</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Dolomite + Bio NPK</t>
+          <t>Ammonium Sulphate + Gypsum</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>pH 0.932</t>
+          <t>pH 8.1</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>, Rain 15.0mm</t>
+          <t>, Rain 354.0mm</t>
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Dolomite + Bio NPK</t>
+          <t>Ammonium Sulphate + Gypsum</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Broadcast + incorporation</t>
+          <t>Soil application</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -3442,40 +3430,40 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>Apply lime to correct pH, then balanced NPK</t>
+          <t>Apply sulfur-based amendments to reduce pH</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Black Wheat</t>
+          <t>Bell Pepper</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>MOP (Potassium-rich)</t>
+          <t>Balanced NPK (15-15-15)</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>N/A, P 97.5, K 52.5</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>, Rain 233.1mm</t>
+          <t>, Rain 16.5mm</t>
         </is>
       </c>
       <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr">
         <is>
-          <t>MOP (Potassium-rich)</t>
+          <t>Balanced NPK (15-15-15)</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Soil application</t>
+          <t>Broadcast + incorporation</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -3484,18 +3472,18 @@
         </is>
       </c>
       <c r="I71" t="n">
-        <v>0.65</v>
+        <v>0.75</v>
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>Increase potassium</t>
+          <t>Maintain current balanced fertilization</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Barley</t>
+          <t>Black Wheat</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3508,8 +3496,14 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr"/>
-      <c r="E72" t="inlineStr"/>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>, Rain 48.0mm</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>5.46</v>
+      </c>
       <c r="F72" t="inlineStr">
         <is>
           <t>Balanced NPK (15-15-15)</t>
@@ -3522,7 +3516,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Every 25-30 days</t>
+          <t>Every 15-20 days</t>
         </is>
       </c>
       <c r="I72" t="n">
@@ -3537,46 +3531,1874 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Barley</t>
+          <t>Carrot</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Dolomite + Bio NPK</t>
+          <t>Balanced NPK (15-15-15)</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>pH 1.0</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>, Rain 400.0mm</t>
-        </is>
-      </c>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr"/>
       <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Every 25-30 days</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>Maintain current balanced fertilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Barley</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Every 25-30 days</t>
+        </is>
+      </c>
+      <c r="I74" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>Maintain current balanced fertilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Black Wheat</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>MOP (Potassium-rich)</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>N/A, P 20.0, K 5.0</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>, Rain 100.0mm</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>MOP (Potassium-rich)</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Soil application</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Every 15-20 days</t>
+        </is>
+      </c>
+      <c r="I75" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>Increase potassium</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Black Wheat</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
           <t>Dolomite + Bio NPK</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>Broadcast + incorporation</t>
-        </is>
-      </c>
-      <c r="H73" t="inlineStr">
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>pH 5.0</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="n">
+        <v>38.18</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Dolomite + Bio NPK</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Every 25-30 days</t>
+        </is>
+      </c>
+      <c r="I76" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>Apply lime to correct pH, then balanced NPK</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Chickpea</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="inlineStr"/>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Every 25-30 days</t>
+        </is>
+      </c>
+      <c r="I77" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>Maintain current balanced fertilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Barley</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>, Rain 10.0mm</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
         <is>
           <t>Every 15-20 days</t>
         </is>
       </c>
-      <c r="I73" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="J73" t="inlineStr">
+      <c r="I78" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>Maintain current balanced fertilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Black Wheat</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>pH 7.7, OC 1.0%</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>, Rain 146.0mm</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Every 15-20 days</t>
+        </is>
+      </c>
+      <c r="I79" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>Maintain current balanced fertilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Barley</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>, Rain 400.0mm</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Every 15-20 days</t>
+        </is>
+      </c>
+      <c r="I80" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>Maintain current balanced fertilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Barley</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>, Rain 485.0mm</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Every 15-20 days</t>
+        </is>
+      </c>
+      <c r="I81" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>Maintain current balanced fertilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Barley</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Dolomite + Bio NPK</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>pH 4.5</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Dolomite + Bio NPK</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Every 25-30 days</t>
+        </is>
+      </c>
+      <c r="I82" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J82" t="inlineStr">
         <is>
           <t>Apply lime to correct pH, then balanced NPK</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Chickpea</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>, Rain 0.0mm</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Every 15-20 days</t>
+        </is>
+      </c>
+      <c r="I83" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>Maintain current balanced fertilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Chickpea</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>, Rain 15.0mm</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Every 15-20 days</t>
+        </is>
+      </c>
+      <c r="I84" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>Maintain current balanced fertilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Barley</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>, Rain 150.0mm</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr"/>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Every 15-20 days</t>
+        </is>
+      </c>
+      <c r="I85" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>Maintain current balanced fertilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Black Wheat</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>MOP (Potassium-rich)</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>N/A, P 97.5, K 52.5</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>, Rain 233.1mm</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>MOP (Potassium-rich)</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Soil application</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Every 15-20 days</t>
+        </is>
+      </c>
+      <c r="I86" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>Increase potassium</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Cotton</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>pH 8.0</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>, Rain 415.49mm</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Every 15-20 days</t>
+        </is>
+      </c>
+      <c r="I87" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>Maintain current balanced fertilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Spinach</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr"/>
+      <c r="E88" t="inlineStr"/>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Every 25-30 days</t>
+        </is>
+      </c>
+      <c r="I88" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>Maintain current balanced fertilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Barley</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>pH 7.06</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>, Rain 600.0mm</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>43.26</v>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Every 25-30 days</t>
+        </is>
+      </c>
+      <c r="I89" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>Maintain current balanced fertilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Bell Pepper</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>MOP (Potassium-rich)</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>pH 5.7, K 46.0</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>, Rain 100.0mm</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>MOP (Potassium-rich)</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Soil application</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Every 15-20 days</t>
+        </is>
+      </c>
+      <c r="I90" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Increase potassium</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Chickpea</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>, Rain 145.12mm</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Every 15-20 days</t>
+        </is>
+      </c>
+      <c r="I91" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>Maintain current balanced fertilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Cabbage</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Dolomite + Bio NPK</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>pH 4.5</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="n">
+        <v>722.89</v>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Dolomite + Bio NPK</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Every 25-30 days</t>
+        </is>
+      </c>
+      <c r="I92" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Apply lime to correct pH, then balanced NPK</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Chickpea</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>, Rain 90.0mm</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Every 15-20 days</t>
+        </is>
+      </c>
+      <c r="I93" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>Maintain current balanced fertilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Barley</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr"/>
+      <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Every 25-30 days</t>
+        </is>
+      </c>
+      <c r="I94" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>Maintain current balanced fertilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Cabbage</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>DAP (Phosphorus-rich)</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>pH 4.56, P 0.0, K 1.0</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr"/>
+      <c r="E95" t="n">
+        <v>14.37</v>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>DAP (Phosphorus-rich)</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Soil application at sowing</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Every 25-30 days</t>
+        </is>
+      </c>
+      <c r="I95" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>Increase phosphorus</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Chickpea</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr"/>
+      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Every 25-30 days</t>
+        </is>
+      </c>
+      <c r="I96" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>Maintain current balanced fertilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Bell Pepper</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>DAP (Phosphorus-rich)</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>pH 5.98, P 2.23, K 1.0</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>, Rain 829.2mm</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>DAP (Phosphorus-rich)</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Soil application at sowing</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Every 25-30 days</t>
+        </is>
+      </c>
+      <c r="I97" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>Increase phosphorus</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Barley</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>, Rain 2021.0mm</t>
+        </is>
+      </c>
+      <c r="E98" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Split application (3-4 splits)</t>
+        </is>
+      </c>
+      <c r="I98" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>Maintain current balanced fertilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Black Wheat</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>, Rain 281.0mm</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Every 15-20 days</t>
+        </is>
+      </c>
+      <c r="I99" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>Maintain current balanced fertilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Black Wheat</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>, Rain 820.0mm</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Every 25-30 days</t>
+        </is>
+      </c>
+      <c r="I100" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>Maintain current balanced fertilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Chickpea</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>pH 6.5</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>, Rain 681.0mm</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Every 25-30 days</t>
+        </is>
+      </c>
+      <c r="I101" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>Maintain current balanced fertilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Chickpea</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>pH 7.9</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr"/>
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Every 25-30 days</t>
+        </is>
+      </c>
+      <c r="I102" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>Maintain current balanced fertilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Black Wheat</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>pH 6.1</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr"/>
+      <c r="E103" t="inlineStr"/>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Every 25-30 days</t>
+        </is>
+      </c>
+      <c r="I103" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>Maintain current balanced fertilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Barley</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>pH 7.0</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>, Rain 986.24mm</t>
+        </is>
+      </c>
+      <c r="E104" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Every 25-30 days</t>
+        </is>
+      </c>
+      <c r="I104" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>Maintain current balanced fertilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Barley</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>pH 5.8</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr"/>
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Every 25-30 days</t>
+        </is>
+      </c>
+      <c r="I105" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>Maintain current balanced fertilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Bell Pepper</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr"/>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Every 25-30 days</t>
+        </is>
+      </c>
+      <c r="I106" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>Maintain current balanced fertilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Bell Pepper</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>, Rain 1369.6mm</t>
+        </is>
+      </c>
+      <c r="E107" t="n">
+        <v>14.97</v>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Split application (3-4 splits)</t>
+        </is>
+      </c>
+      <c r="I107" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>Maintain current balanced fertilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Bell Pepper</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>pH 6.8</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr"/>
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>Every 25-30 days</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>Maintain current balanced fertilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Maize</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>pH 7.88, OC 8.0%</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr"/>
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>Every 25-30 days</t>
+        </is>
+      </c>
+      <c r="I109" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>Maintain current balanced fertilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Chickpea</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr"/>
+      <c r="E110" t="n">
+        <v>331.2</v>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>Every 25-30 days</t>
+        </is>
+      </c>
+      <c r="I110" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>Maintain current balanced fertilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Chickpea</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>pH 7.3</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr"/>
+      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>Every 25-30 days</t>
+        </is>
+      </c>
+      <c r="I111" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>Maintain current balanced fertilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Chickpea</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>pH 6.7</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr"/>
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>Every 25-30 days</t>
+        </is>
+      </c>
+      <c r="I112" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>Maintain current balanced fertilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Black Wheat</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>, Rain 100.0mm</t>
+        </is>
+      </c>
+      <c r="E113" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>Every 15-20 days</t>
+        </is>
+      </c>
+      <c r="I113" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>Maintain current balanced fertilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Barley</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>N/A, OC 0.5232%</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr"/>
+      <c r="E114" t="inlineStr"/>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Balanced NPK (15-15-15)</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>Broadcast + incorporation</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>Every 25-30 days</t>
+        </is>
+      </c>
+      <c r="I114" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>Maintain current balanced fertilization</t>
         </is>
       </c>
     </row>

</xml_diff>